<commit_message>
Scalars in dump file processing
</commit_message>
<xml_diff>
--- a/results/2030_BS0001/Sankey_sequences_all_scenarios.xlsx
+++ b/results/2030_BS0001/Sankey_sequences_all_scenarios.xlsx
@@ -9,7 +9,8 @@
   <sheets>
     <sheet name="Main_Sheet" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="2030_BS0001_001" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="2030_BS0001_ref" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="2030_BS0001_002" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="2030_BS0001_ref" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -13293,7 +13294,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="B3" showErrorMessage="1" showDropDown="0" showInputMessage="1" allowBlank="0" type="list">
-      <formula1>"2030_BS0001_001,2030_BS0001_ref"</formula1>
+      <formula1>"2030_BS0001_001,2030_BS0001_002,2030_BS0001_ref"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -16962,7 +16963,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2030_BS0001_ref</t>
+          <t>2030_BS0001_002</t>
         </is>
       </c>
     </row>
@@ -16978,7 +16979,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>9252.200420210362</v>
+        <v>4051583.584138229</v>
       </c>
     </row>
     <row r="8">
@@ -16988,7 +16989,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>4492641.862961633</v>
       </c>
     </row>
     <row r="9">
@@ -16998,7 +16999,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>12813455.68516653</v>
+        <v>12718669.25987154</v>
       </c>
     </row>
     <row r="10">
@@ -17008,7 +17009,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1379.032203261238</v>
+        <v>575661.6793061675</v>
       </c>
     </row>
     <row r="11">
@@ -17018,7 +17019,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>11032257.62608992</v>
+        <v>460529.3434449342</v>
       </c>
     </row>
     <row r="12">
@@ -17088,6 +17089,3643 @@
         </is>
       </c>
       <c r="D22" t="n">
+        <v>6056273.000000016</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Bioholz</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Bioholz Bus</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Biomasse - Kraftwerk</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Bioholz</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Bioholz Bus</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Biomasse - Heizkraftwerk</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Bioholz</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Bioholz Bus</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Biomasse - Heizwerk</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Bioholz</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Biomasse - Holz</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Bioholz Bus</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>6056273.000000016</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Biomass</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Biomass Bus</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Biogas-BHKW</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>2784930.999999999</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Biomass</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Biomass Bus</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Biogasaufbereitunganlage</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Biomass</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Biomass Bus</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Biomethaneinspeisungsanlage</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Biomass</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Biomass Bus</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Biomass to Liquid</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Biomass</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Biomass Bus</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>excess_b_bio</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Biomass</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Biomasse - Substrat</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Biomass Bus</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>2784930.999999999</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Fernwaerme</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Fernwaerme Bus</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Fernwaermespeicher</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>883123.4116396789</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Fernwaerme</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Fernwaerme Bus</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Saisonaler Waermespeicher</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Fernwaerme</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Fernwaerme Bus</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Heat_demand_total</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>3126015.419637652</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Fernwaerme</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Fernwaerme Bus</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>excess_b_distheat</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>0</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Fernwaerme</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Biogas-BHKW</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Fernwaerme Bus</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>1364616.19</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Fernwaerme</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Biomasse - Heizkraftwerk</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Fernwaerme Bus</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Fernwaerme</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Biomasse - Heizwerk</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Fernwaerme Bus</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>0</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Fernwaerme</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Elektodenheizstab</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Fernwaerme Bus</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>946637.7761366254</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Fernwaerme</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>GuD in KWK</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Fernwaerme Bus</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>842154.7607696985</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Fernwaerme</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Fernwaermespeicher</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Fernwaerme Bus</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>855730.1043710072</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Fernwaerme</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Luft-Waermepumpe</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Fernwaerme Bus</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>0</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Fernwaerme</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Abwaerme-Waermepumpe</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Fernwaerme Bus</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>0</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Fernwaerme</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Erd-Waermepumpe</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Fernwaerme Bus</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>0</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Fernwaerme</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Nachheizung - Heizstab</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Fernwaerme Bus</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>0</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Fernwaerme</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Nachheizung - WP</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Fernwaerme Bus</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>0</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Fernwaerme</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Solarthermie</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Fernwaerme Bus</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>0</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Strom</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Strom Bus</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Batteriespeicher</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>916290.8921442947</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Strom</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Strom Bus</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Elektodenheizstab</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>956199.7738753791</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Strom</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Strom Bus</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Electricity_demand_total</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>12509397.49112029</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Strom</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Strom Bus</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Elektrolyse</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>2843238.026186052</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Strom</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Strom Bus</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Export_Electricity</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>6882167.380356727</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Strom</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Strom Bus</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Luft-Waermepumpe</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>0</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Strom</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Strom Bus</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Abwaerme-Waermepumpe</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>0</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Strom</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Strom Bus</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Erd-Waermepumpe</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>0</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Strom</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Strom Bus</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Hös&lt;-&gt;HS</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>0</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Strom</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Strom Bus</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Nachheizung - Heizstab</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>0</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Strom</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Strom Bus</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Nachheizung - WP</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>0</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Strom</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Strom Bus</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Power to Liquid</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>0</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Strom</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Strom Bus</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Pumpspeicherkraftwerk</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>575661.6793061675</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Strom</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Strom Bus</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>excess_b_el</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>0</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Strom</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Batteriespeicher</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Strom Bus</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>824661.8029298653</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Strom</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Biogas-BHKW</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Strom Bus</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>1058273.78</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Strom</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Biomasse - Kraftwerk</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Strom Bus</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>0</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Strom</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Biomasse - Heizkraftwerk</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Strom Bus</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>0</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Strom</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Brennstoffzelle</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Strom Bus</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>0</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Strom</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>GuD in KWK</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Strom Bus</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>881324.7496427079</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Strom</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Wasserkraft</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Strom Bus</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>195270.86</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Strom</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Hös&lt;-&gt;HS</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Strom Bus</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>4051583.584138229</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Strom</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>PV_open_east</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Strom Bus</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>1055691.873717548</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Strom</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>PV_open_middle</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Strom Bus</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>1081045.962526691</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Strom</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>PV_open_north</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Strom Bus</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>797447.6565784265</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Strom</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>PV_open_swest</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Strom Bus</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>1558456.370138968</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Strom</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>PV_rooftop_east</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Strom Bus</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>0</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Strom</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>PV_rooftop_middle</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Strom Bus</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>0</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Strom</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>PV_rooftop_north</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Strom Bus</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>0</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Strom</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>PV_rooftop_swest</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Strom Bus</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>0</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Strom</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Pumpspeicherkraftwerk</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Strom Bus</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>460529.3434449342</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Strom</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Wind_east</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Strom Bus</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>4111777.52773424</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Strom</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Wind_middle</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Strom Bus</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>3756028.42636268</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Strom</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Wind_north</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Strom Bus</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>2781520.71112652</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Strom</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Wind_swest</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Strom Bus</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>2069342.5946481</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="102"/>
+    <row r="103"/>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Electricity_Hös</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Electricity_Hös Bus</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Hös&lt;-&gt;HS</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>4051583.584138229</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Electricity_Hös</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Electricity_Hös Bus</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Pumpspeicherkraftwerk - Goldistal</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>0</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Electricity_Hös</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Hös&lt;-&gt;HS</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Electricity_Hös Bus</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>0</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Electricity_Hös</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Import - Stromboerse</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Electricity_Hös Bus</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>4051583.584138229</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Electricity_Hös</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Pumpspeicherkraftwerk - Goldistal</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Electricity_Hös Bus</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>0</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="113"/>
+    <row r="114"/>
+    <row r="115"/>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Umweltwaerme</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Umweltwaerme Bus</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Erd-Waermepumpe</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>0</v>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Umweltwaerme</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Umweltwaerme</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Umweltwaerme Bus</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>0</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="121"/>
+    <row r="122"/>
+    <row r="123"/>
+    <row r="124"/>
+    <row r="125"/>
+    <row r="126"/>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Gas</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Gas Bus</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Gas_demand_total</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>9405355.157340698</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Gas</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Gas Bus</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Erdgasspeicher</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>0</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Gas</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Gas Bus</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>GuD in KWK</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>1958499.443650462</v>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Gas</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Gas Bus</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Material_demand_Gas</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>27774.6067985753</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Gas</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Gas Bus</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>excess_b_gas</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>0</v>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Gas</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Biogasaufbereitunganlage</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Gas Bus</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>0</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Gas</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Biomethaneinspeisungsanlage</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Gas Bus</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>0</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Gas</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Erdgasspeicher</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Gas Bus</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>0</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Gas</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Wasserstoff-Einspeisung</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Gas Bus</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>0</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Gas</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Import - Gasnetz</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Gas Bus</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>11391629.20778973</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Gas</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Methanisierung</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Gas Bus</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>0</v>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="138"/>
+    <row r="139"/>
+    <row r="140"/>
+    <row r="141"/>
+    <row r="142"/>
+    <row r="143"/>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Wassterstoff</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Wassterstoff Bus</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Export_Hydrogen</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>2388319.941996283</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Wassterstoff</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Wassterstoff Bus</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Brennstoffzelle</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>0</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Wassterstoff</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Wassterstoff Bus</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Wasserstoffspeicher</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>0</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Wassterstoff</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Wassterstoff Bus</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Hydrogen_demand_total</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>0</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Wassterstoff</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Wassterstoff Bus</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Wasserstoff-Einspeisung</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>0</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Wassterstoff</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Wassterstoff Bus</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Methanisierung</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>0</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Wassterstoff</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Wassterstoff Bus</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Power to Liquid</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>0</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Wassterstoff</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Wassterstoff Bus</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>excess_b_H2</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>0</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Wassterstoff</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Elektrolyse</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Wassterstoff Bus</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>2388319.941996283</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Wassterstoff</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Wasserstoffspeicher</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Wassterstoff Bus</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>0</v>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Wassterstoff</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Import - Wasserstoff</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Wassterstoff Bus</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>0</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="155"/>
+    <row r="156"/>
+    <row r="157"/>
+    <row r="158"/>
+    <row r="159"/>
+    <row r="160"/>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Oel&amp;Kraftstoff</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Oel&amp;Kraftstoff Bus</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Material_demand_Oil</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>1138758.878741587</v>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Oel&amp;Kraftstoff</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Oel&amp;Kraftstoff Bus</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Oil &amp; fuel_demand_total</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>11009033.27980609</v>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Oel&amp;Kraftstoff</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Oel&amp;Kraftstoff Bus</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>excess_b_oil_fuel</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>0</v>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Oel&amp;Kraftstoff</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Biomass to Liquid</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Oel&amp;Kraftstoff Bus</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>0</v>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>Oel&amp;Kraftstoff</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Import - Heizoel &amp; Kraftstoffe</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Oel&amp;Kraftstoff Bus</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>12147792.15854768</v>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Oel&amp;Kraftstoff</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Import - Synth. Kraftstoffe</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Oel&amp;Kraftstoff Bus</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>0</v>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>Oel&amp;Kraftstoff</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Power to Liquid</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Oel&amp;Kraftstoff Bus</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>0</v>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Nachheizung</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Nachheizung Bus</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Nachheizung - Heizstab</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>0</v>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Nachheizung</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Nachheizung Bus</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Nachheizung - WP</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>0</v>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Nachheizung</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Saisonaler Waermespeicher</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Nachheizung Bus</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>0</v>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>Abwaerme</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Abwaerme Bus</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Abwaerme-Waermepumpe</t>
+        </is>
+      </c>
+      <c r="D183" t="n">
+        <v>0</v>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>Abwaerme</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>AW</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Abwaerme Bus</t>
+        </is>
+      </c>
+      <c r="D184" t="n">
+        <v>0</v>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>Festbrennstoff</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Festbrennstoff Bus</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Biomass_demand_total</t>
+        </is>
+      </c>
+      <c r="D191" t="n">
+        <v>6470967.58864251</v>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>Bus sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>Festbrennstoff</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Biomasse als Festbrennstoff</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Festbrennstoff Bus</t>
+        </is>
+      </c>
+      <c r="D192" t="n">
+        <v>6056273.000000016</v>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>Festbrennstoff</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Import - Braunkohle</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Festbrennstoff Bus</t>
+        </is>
+      </c>
+      <c r="D193" t="n">
+        <v>0</v>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>Festbrennstoff</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Import - Steinkohle</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Festbrennstoff Bus</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>414694.5886424932</v>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
+    <row r="200"/>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Batteriespeicher</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>None Bus</t>
+        </is>
+      </c>
+      <c r="D201" t="n">
+        <v>0</v>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Erdgasspeicher</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>None Bus</t>
+        </is>
+      </c>
+      <c r="D202" t="n">
+        <v>0</v>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Wasserstoffspeicher</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>None Bus</t>
+        </is>
+      </c>
+      <c r="D203" t="n">
+        <v>0</v>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Fernwaermespeicher</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>None Bus</t>
+        </is>
+      </c>
+      <c r="D204" t="n">
+        <v>0</v>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Saisonaler Waermespeicher</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>None Bus</t>
+        </is>
+      </c>
+      <c r="D205" t="n">
+        <v>0</v>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Pumpspeicherkraftwerk</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>None Bus</t>
+        </is>
+      </c>
+      <c r="D206" t="n">
+        <v>0</v>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Pumpspeicherkraftwerk - Goldistal</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>None Bus</t>
+        </is>
+      </c>
+      <c r="D207" t="n">
+        <v>0</v>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>MWh</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>Component sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="208"/>
+    <row r="209"/>
+    <row r="210"/>
+    <row r="211"/>
+    <row r="212"/>
+    <row r="213"/>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F213"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Basic_example_zorro_1</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>2030_BS0001_ref</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4"/>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Import Strom flow</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>9252.200420210362</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Total PV Flow</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Total Wind Flow</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>12813455.68516653</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Total Pumpspeicher Eingangsflow</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1379.032203261238</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Total Pumpspeicher Ausgangsflow</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>11032257.62608992</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Umweltwaermemenge_Luft_waermepumpe</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>Bus</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="C21" s="1" t="inlineStr">
+        <is>
+          <t>To</t>
+        </is>
+      </c>
+      <c r="D21" s="1" t="inlineStr">
+        <is>
+          <t>Flow</t>
+        </is>
+      </c>
+      <c r="E21" s="1" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="F21" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Bioholz</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Bioholz Bus</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Biomasse als Festbrennstoff</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
         <v>5937790.22766629</v>
       </c>
       <c r="E22" t="inlineStr">

</xml_diff>